<commit_message>
Update dateien.json, audio und noten
</commit_message>
<xml_diff>
--- a/besetzung.xlsx
+++ b/besetzung.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://thaddenschulede-my.sharepoint.com/personal/lepold_thaddenschule_de/Documents/12 GitHub/thadden27/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{1CF0D39D-5D34-4E0C-B484-DB3499A4EFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EC8EB2C-74DE-45AC-8A02-83CA26A31791}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{1CF0D39D-5D34-4E0C-B484-DB3499A4EFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8298BDB7-B958-4D8B-96FC-6112A53657EE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{870A77A3-6497-424F-BFDB-56D4CBDBF5BF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{870A77A3-6497-424F-BFDB-56D4CBDBF5BF}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="101">
   <si>
     <t>Szene</t>
   </si>
@@ -194,9 +194,6 @@
     <t xml:space="preserve">Dystopie </t>
   </si>
   <si>
-    <t>Mögliches Happy End</t>
-  </si>
-  <si>
     <t>Finale</t>
   </si>
   <si>
@@ -326,9 +323,6 @@
     <t>13</t>
   </si>
   <si>
-    <t>Ermordung Elisabeth "Mach End o Herr"</t>
-  </si>
-  <si>
     <t>12.1</t>
   </si>
   <si>
@@ -338,13 +332,13 @@
     <t>12.3</t>
   </si>
   <si>
-    <t>12.4</t>
-  </si>
-  <si>
     <t>8.2</t>
   </si>
   <si>
     <t>9.1</t>
+  </si>
+  <si>
+    <t>Ermordung Elisabeth "Mach End o Herr" (acappella)</t>
   </si>
 </sst>
 </file>
@@ -860,7 +854,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EAA9A49-82B2-433C-BF39-5078DFD427BF}">
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" style="25"/>
@@ -891,13 +885,13 @@
         <v>25</v>
       </c>
       <c r="E1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F1" t="s">
         <v>30</v>
       </c>
       <c r="G1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H1" s="5" t="s">
         <v>2</v>
@@ -929,7 +923,7 @@
         <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>19</v>
@@ -950,7 +944,7 @@
         <v>19</v>
       </c>
       <c r="G3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="N3" t="s">
         <v>19</v>
@@ -981,7 +975,7 @@
         <v>19</v>
       </c>
       <c r="G5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J5" s="10" t="s">
         <v>19</v>
@@ -1017,7 +1011,7 @@
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H7" s="7"/>
       <c r="J7" s="8"/>
@@ -1042,7 +1036,7 @@
       <c r="E8" s="21"/>
       <c r="F8" s="21"/>
       <c r="G8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H8" s="9" t="s">
         <v>19</v>
@@ -1097,10 +1091,10 @@
         <v>27</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H11" s="9" t="s">
         <v>19</v>
@@ -1123,7 +1117,7 @@
         <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F12" t="s">
         <v>19</v>
@@ -1137,7 +1131,7 @@
         <v>31</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>19</v>
@@ -1152,16 +1146,16 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>19</v>
       </c>
       <c r="G14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>19</v>
@@ -1172,10 +1166,10 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="25" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>19</v>
@@ -1186,16 +1180,16 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" t="s">
         <v>72</v>
       </c>
-      <c r="B16" t="s">
-        <v>73</v>
-      </c>
       <c r="C16" s="9" t="s">
         <v>19</v>
       </c>
       <c r="G16" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>19</v>
@@ -1209,10 +1203,10 @@
     </row>
     <row r="17" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="26" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C17" s="7"/>
       <c r="D17" s="8" t="s">
@@ -1227,10 +1221,10 @@
     </row>
     <row r="18" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="26" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>19</v>
@@ -1242,7 +1236,7 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B19" t="s">
         <v>34</v>
@@ -1256,10 +1250,10 @@
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="25" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B20" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>19</v>
@@ -1268,7 +1262,7 @@
         <v>19</v>
       </c>
       <c r="G20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="L20" t="s">
         <v>19</v>
@@ -1319,7 +1313,7 @@
         <v>19</v>
       </c>
       <c r="G23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M23" t="s">
         <v>19</v>
@@ -1345,7 +1339,7 @@
         <v>19</v>
       </c>
       <c r="G24" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I24" t="s">
         <v>19</v>
@@ -1365,7 +1359,7 @@
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="25" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B25" t="s">
         <v>42</v>
@@ -1377,7 +1371,7 @@
         <v>19</v>
       </c>
       <c r="G25" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K25" t="s">
         <v>19</v>
@@ -1388,7 +1382,7 @@
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="25" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B26" t="s">
         <v>43</v>
@@ -1400,7 +1394,7 @@
         <v>19</v>
       </c>
       <c r="G26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I26" t="s">
         <v>19</v>
@@ -1417,7 +1411,7 @@
         <v>37</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>19</v>
@@ -1435,7 +1429,7 @@
         <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C28" s="9" t="s">
         <v>19</v>
@@ -1449,10 +1443,10 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="25" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B29" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C29" s="9" t="s">
         <v>19</v>
@@ -1466,7 +1460,7 @@
         <v>44</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C30" s="7"/>
       <c r="D30" s="8" t="s">
@@ -1478,10 +1472,10 @@
     </row>
     <row r="31" spans="1:15" s="28" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="25" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B31" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C31" s="29"/>
       <c r="D31" s="30" t="s">
@@ -1491,7 +1485,7 @@
         <v>19</v>
       </c>
       <c r="G31" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H31" s="29"/>
       <c r="J31" s="30" t="s">
@@ -1507,7 +1501,7 @@
         <v>45</v>
       </c>
       <c r="B32" s="32" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C32" s="33" t="s">
         <v>19</v>
@@ -1525,7 +1519,7 @@
         <v>46</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C33" s="7"/>
       <c r="D33" s="8" t="s">
@@ -1537,10 +1531,10 @@
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="25" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B34" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D34" s="10" t="s">
         <v>19</v>
@@ -1548,13 +1542,13 @@
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="25" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B35" s="24" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G35" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H35" s="9" t="s">
         <v>19</v>
@@ -1574,10 +1568,10 @@
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="25" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B36" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D36" s="10" t="s">
         <v>19</v>
@@ -1614,10 +1608,10 @@
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="25" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B38" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C38" s="9" t="s">
         <v>19</v>
@@ -1626,7 +1620,7 @@
         <v>19</v>
       </c>
       <c r="G38" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H38" s="9" t="s">
         <v>19</v>
@@ -1640,7 +1634,7 @@
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="25" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B39" t="s">
         <v>51</v>
@@ -1654,10 +1648,10 @@
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="25" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B40" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D40" s="10" t="s">
         <v>19</v>
@@ -1672,51 +1666,37 @@
         <v>19</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A41" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="B41" t="s">
+    <row r="41" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="26" t="s">
+        <v>94</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="F41" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="42" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="26" t="s">
-        <v>95</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C42" s="7"/>
-      <c r="D42" s="8"/>
-      <c r="G42" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="H42" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="I42" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="J42" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="L42" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="M42" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="N42" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="O42" s="7" t="s">
+      <c r="C41" s="7"/>
+      <c r="D41" s="8"/>
+      <c r="G41" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="H41" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="I41" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J41" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="L41" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M41" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N41" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O41" s="7" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>